<commit_message>
Corregir dos notas que Excel interpretaria como formula y verificar el libro
Dos celdas de texto empezaban por '=', lo que Excel habria evaluado como
formula. Se reformulan.

Se anade scripts/verificar_modelo.py, que evalua las 997 celdas del libro
con la libreria formulas y contrasta 26 cifras clave localizando cada
celda por su etiqueta. Resultado: 0 errores de formula, 0 desviaciones.
LibreOffice no es viable en este entorno (no recalcula ni un archivo de
tres celdas en 4 minutos), de ahi la verificacion alternativa.
</commit_message>
<xml_diff>
--- a/Alcopalet_Modelo_Financiero.xlsx
+++ b/Alcopalet_Modelo_Financiero.xlsx
@@ -907,7 +907,7 @@
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>Utilización actual de la fábrica</t>
+          <t>Capacidad anual actual (palets)</t>
         </is>
       </c>
       <c r="B27" s="11">
@@ -916,7 +916,7 @@
       </c>
       <c r="C27" s="9" t="inlineStr">
         <is>
-          <t>Capacidad anual frente a 174.504 palets producidos: la fábrica está al 81%.</t>
+          <t>Frente a 174.504 palets producidos en 2025: la fábrica está al 81%, no llena.</t>
         </is>
       </c>
     </row>
@@ -3306,9 +3306,10 @@
         <f>Escandallo!$B$7*Lineas!$B$7/Datos!$B$9</f>
         <v/>
       </c>
-      <c r="F23" s="9">
-        <f> 10 operarios: los 8 de manual + los 2 de la línea automática. Coherente.</f>
-        <v/>
+      <c r="F23" s="9" t="inlineStr">
+        <is>
+          <t>Da 10 operarios: los 8 de manual más los 2 de la línea automática. Coherente.</t>
+        </is>
       </c>
     </row>
     <row r="24">
@@ -3321,9 +3322,10 @@
         <f>Escandallo!$C$7*Lineas!$C$7/Datos!$B$9</f>
         <v/>
       </c>
-      <c r="F24" s="9">
-        <f> 7 operarios. Coincide exactamente con el dato del caso. El escandallo es fiable.</f>
-        <v/>
+      <c r="F24" s="9" t="inlineStr">
+        <is>
+          <t>Da 7 operarios. Coincide exactamente con el dato del caso: el escandallo es fiable.</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -4747,7 +4749,7 @@
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
-          <t>Comprobación: el resultado del robot coincide con los 0,42 €/ud del Anexo 3.</t>
+          <t>Coste a plena capacidad de cada sistema. No coincide con el Anexo 3 (2,18 € y 0,42 €) porque el anexo promedia manual y línea automática, y porque atribuye al robot 90.000 unidades cuando su capacidad real es de 87.120.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Inyectar los valores calculados en los libros para que se vean sin recalcular
openpyxl escribe las formulas sin valor cacheado, asi que los visores
(movil, vista previa, Excel Online) mostraban las celdas en blanco.

Se anade scripts/inyectar_valores.py, que evalua el libro y escribe el
resultado como <v> dentro del XML conservando la formula. Corrige ademas
tres fallos propios: el orden de atributos en workbook.xml.rels, la barra
inicial del Target, y las celdas vacias autocerradas, que el patron se
tragaba junto con la celda siguiente.

Resultado: 70 y 331 formulas respectivamente, ninguna sin valor visible.
</commit_message>
<xml_diff>
--- a/Alcopalet_Modelo_Financiero.xlsx
+++ b/Alcopalet_Modelo_Financiero.xlsx
@@ -864,7 +864,7 @@
       </c>
       <c r="B24" s="8">
         <f>Escandallo!$D$11</f>
-        <v/>
+        <v>-0.5199999999999996</v>
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
@@ -880,7 +880,7 @@
       </c>
       <c r="B25" s="10">
         <f>Persan!$B$19</f>
-        <v/>
+        <v>-188876.67123287672</v>
       </c>
       <c r="C25" s="9" t="inlineStr">
         <is>
@@ -896,7 +896,7 @@
       </c>
       <c r="B26" s="8">
         <f>Persan!$B$28</f>
-        <v/>
+        <v>12.170128022759602</v>
       </c>
       <c r="C26" s="9" t="inlineStr">
         <is>
@@ -912,7 +912,7 @@
       </c>
       <c r="B27" s="11">
         <f>Capacidad!$D$8</f>
-        <v/>
+        <v>215380.0</v>
       </c>
       <c r="C27" s="9" t="inlineStr">
         <is>
@@ -928,7 +928,7 @@
       </c>
       <c r="B28" s="10">
         <f>PyG2025!$B$31</f>
-        <v/>
+        <v>-60555.0</v>
       </c>
       <c r="C28" s="9" t="inlineStr">
         <is>
@@ -1087,35 +1087,35 @@
       </c>
       <c r="B6" s="68">
         <f>Datos!$B$14*(B$4-(Escandallo!$D$6*(1+$A6)+Escandallo!$D$7+Escandallo!$D$8+Escandallo!$D$9))-Datos!$B$50-Datos!$B$53-(B$4*Datos!$B$14*Datos!$B$17/365+Datos!$B$18*Escandallo!$D$10)*Datos!$B$11</f>
-        <v/>
+        <v>-151661.67123287675</v>
       </c>
       <c r="C6" s="68">
         <f>Datos!$B$14*(C$4-(Escandallo!$D$6*(1+$A6)+Escandallo!$D$7+Escandallo!$D$8+Escandallo!$D$9))-Datos!$B$50-Datos!$B$53-(C$4*Datos!$B$14*Datos!$B$17/365+Datos!$B$18*Escandallo!$D$10)*Datos!$B$11</f>
-        <v/>
+        <v>-108326.05479452059</v>
       </c>
       <c r="D6" s="68">
         <f>Datos!$B$14*(D$4-(Escandallo!$D$6*(1+$A6)+Escandallo!$D$7+Escandallo!$D$8+Escandallo!$D$9))-Datos!$B$50-Datos!$B$53-(D$4*Datos!$B$14*Datos!$B$17/365+Datos!$B$18*Escandallo!$D$10)*Datos!$B$11</f>
-        <v/>
+        <v>-64990.43835616443</v>
       </c>
       <c r="E6" s="68">
         <f>Datos!$B$14*(E$4-(Escandallo!$D$6*(1+$A6)+Escandallo!$D$7+Escandallo!$D$8+Escandallo!$D$9))-Datos!$B$50-Datos!$B$53-(E$4*Datos!$B$14*Datos!$B$17/365+Datos!$B$18*Escandallo!$D$10)*Datos!$B$11</f>
-        <v/>
+        <v>-21654.821917808265</v>
       </c>
       <c r="F6" s="68">
         <f>Datos!$B$14*(F$4-(Escandallo!$D$6*(1+$A6)+Escandallo!$D$7+Escandallo!$D$8+Escandallo!$D$9))-Datos!$B$50-Datos!$B$53-(F$4*Datos!$B$14*Datos!$B$17/365+Datos!$B$18*Escandallo!$D$10)*Datos!$B$11</f>
-        <v/>
+        <v>21680.79452054792</v>
       </c>
       <c r="G6" s="68">
         <f>Datos!$B$14*(G$4-(Escandallo!$D$6*(1+$A6)+Escandallo!$D$7+Escandallo!$D$8+Escandallo!$D$9))-Datos!$B$50-Datos!$B$53-(G$4*Datos!$B$14*Datos!$B$17/365+Datos!$B$18*Escandallo!$D$10)*Datos!$B$11</f>
-        <v/>
+        <v>65016.41095890408</v>
       </c>
       <c r="H6" s="68">
         <f>Datos!$B$14*(H$4-(Escandallo!$D$6*(1+$A6)+Escandallo!$D$7+Escandallo!$D$8+Escandallo!$D$9))-Datos!$B$50-Datos!$B$53-(H$4*Datos!$B$14*Datos!$B$17/365+Datos!$B$18*Escandallo!$D$10)*Datos!$B$11</f>
-        <v/>
+        <v>108352.02739726024</v>
       </c>
       <c r="I6" s="68">
         <f>Datos!$B$14*(I$4-(Escandallo!$D$6*(1+$A6)+Escandallo!$D$7+Escandallo!$D$8+Escandallo!$D$9))-Datos!$B$50-Datos!$B$53-(I$4*Datos!$B$14*Datos!$B$17/365+Datos!$B$18*Escandallo!$D$10)*Datos!$B$11</f>
-        <v/>
+        <v>151687.64383561639</v>
       </c>
     </row>
     <row r="7">
@@ -1124,35 +1124,35 @@
       </c>
       <c r="B7" s="68">
         <f>Datos!$B$14*(B$4-(Escandallo!$D$6*(1+$A7)+Escandallo!$D$7+Escandallo!$D$8+Escandallo!$D$9))-Datos!$B$50-Datos!$B$53-(B$4*Datos!$B$14*Datos!$B$17/365+Datos!$B$18*Escandallo!$D$10)*Datos!$B$11</f>
-        <v/>
+        <v>-188876.6712328767</v>
       </c>
       <c r="C7" s="68">
         <f>Datos!$B$14*(C$4-(Escandallo!$D$6*(1+$A7)+Escandallo!$D$7+Escandallo!$D$8+Escandallo!$D$9))-Datos!$B$50-Datos!$B$53-(C$4*Datos!$B$14*Datos!$B$17/365+Datos!$B$18*Escandallo!$D$10)*Datos!$B$11</f>
-        <v/>
+        <v>-145541.05479452052</v>
       </c>
       <c r="D7" s="68">
         <f>Datos!$B$14*(D$4-(Escandallo!$D$6*(1+$A7)+Escandallo!$D$7+Escandallo!$D$8+Escandallo!$D$9))-Datos!$B$50-Datos!$B$53-(D$4*Datos!$B$14*Datos!$B$17/365+Datos!$B$18*Escandallo!$D$10)*Datos!$B$11</f>
-        <v/>
+        <v>-102205.43835616435</v>
       </c>
       <c r="E7" s="68">
         <f>Datos!$B$14*(E$4-(Escandallo!$D$6*(1+$A7)+Escandallo!$D$7+Escandallo!$D$8+Escandallo!$D$9))-Datos!$B$50-Datos!$B$53-(E$4*Datos!$B$14*Datos!$B$17/365+Datos!$B$18*Escandallo!$D$10)*Datos!$B$11</f>
-        <v/>
+        <v>-58869.82191780818</v>
       </c>
       <c r="F7" s="68">
         <f>Datos!$B$14*(F$4-(Escandallo!$D$6*(1+$A7)+Escandallo!$D$7+Escandallo!$D$8+Escandallo!$D$9))-Datos!$B$50-Datos!$B$53-(F$4*Datos!$B$14*Datos!$B$17/365+Datos!$B$18*Escandallo!$D$10)*Datos!$B$11</f>
-        <v/>
+        <v>-15534.205479452023</v>
       </c>
       <c r="G7" s="68">
         <f>Datos!$B$14*(G$4-(Escandallo!$D$6*(1+$A7)+Escandallo!$D$7+Escandallo!$D$8+Escandallo!$D$9))-Datos!$B$50-Datos!$B$53-(G$4*Datos!$B$14*Datos!$B$17/365+Datos!$B$18*Escandallo!$D$10)*Datos!$B$11</f>
-        <v/>
+        <v>27801.41095890414</v>
       </c>
       <c r="H7" s="68">
         <f>Datos!$B$14*(H$4-(Escandallo!$D$6*(1+$A7)+Escandallo!$D$7+Escandallo!$D$8+Escandallo!$D$9))-Datos!$B$50-Datos!$B$53-(H$4*Datos!$B$14*Datos!$B$17/365+Datos!$B$18*Escandallo!$D$10)*Datos!$B$11</f>
-        <v/>
+        <v>71137.0273972603</v>
       </c>
       <c r="I7" s="68">
         <f>Datos!$B$14*(I$4-(Escandallo!$D$6*(1+$A7)+Escandallo!$D$7+Escandallo!$D$8+Escandallo!$D$9))-Datos!$B$50-Datos!$B$53-(I$4*Datos!$B$14*Datos!$B$17/365+Datos!$B$18*Escandallo!$D$10)*Datos!$B$11</f>
-        <v/>
+        <v>114472.6438356165</v>
       </c>
     </row>
     <row r="8">
@@ -1161,35 +1161,35 @@
       </c>
       <c r="B8" s="68">
         <f>Datos!$B$14*(B$4-(Escandallo!$D$6*(1+$A8)+Escandallo!$D$7+Escandallo!$D$8+Escandallo!$D$9))-Datos!$B$50-Datos!$B$53-(B$4*Datos!$B$14*Datos!$B$17/365+Datos!$B$18*Escandallo!$D$10)*Datos!$B$11</f>
-        <v/>
+        <v>-226091.67123287678</v>
       </c>
       <c r="C8" s="68">
         <f>Datos!$B$14*(C$4-(Escandallo!$D$6*(1+$A8)+Escandallo!$D$7+Escandallo!$D$8+Escandallo!$D$9))-Datos!$B$50-Datos!$B$53-(C$4*Datos!$B$14*Datos!$B$17/365+Datos!$B$18*Escandallo!$D$10)*Datos!$B$11</f>
-        <v/>
+        <v>-182756.05479452058</v>
       </c>
       <c r="D8" s="68">
         <f>Datos!$B$14*(D$4-(Escandallo!$D$6*(1+$A8)+Escandallo!$D$7+Escandallo!$D$8+Escandallo!$D$9))-Datos!$B$50-Datos!$B$53-(D$4*Datos!$B$14*Datos!$B$17/365+Datos!$B$18*Escandallo!$D$10)*Datos!$B$11</f>
-        <v/>
+        <v>-139420.43835616444</v>
       </c>
       <c r="E8" s="68">
         <f>Datos!$B$14*(E$4-(Escandallo!$D$6*(1+$A8)+Escandallo!$D$7+Escandallo!$D$8+Escandallo!$D$9))-Datos!$B$50-Datos!$B$53-(E$4*Datos!$B$14*Datos!$B$17/365+Datos!$B$18*Escandallo!$D$10)*Datos!$B$11</f>
-        <v/>
+        <v>-96084.82191780827</v>
       </c>
       <c r="F8" s="68">
         <f>Datos!$B$14*(F$4-(Escandallo!$D$6*(1+$A8)+Escandallo!$D$7+Escandallo!$D$8+Escandallo!$D$9))-Datos!$B$50-Datos!$B$53-(F$4*Datos!$B$14*Datos!$B$17/365+Datos!$B$18*Escandallo!$D$10)*Datos!$B$11</f>
-        <v/>
+        <v>-52749.205479452095</v>
       </c>
       <c r="G8" s="68">
         <f>Datos!$B$14*(G$4-(Escandallo!$D$6*(1+$A8)+Escandallo!$D$7+Escandallo!$D$8+Escandallo!$D$9))-Datos!$B$50-Datos!$B$53-(G$4*Datos!$B$14*Datos!$B$17/365+Datos!$B$18*Escandallo!$D$10)*Datos!$B$11</f>
-        <v/>
+        <v>-9413.589041095918</v>
       </c>
       <c r="H8" s="68">
         <f>Datos!$B$14*(H$4-(Escandallo!$D$6*(1+$A8)+Escandallo!$D$7+Escandallo!$D$8+Escandallo!$D$9))-Datos!$B$50-Datos!$B$53-(H$4*Datos!$B$14*Datos!$B$17/365+Datos!$B$18*Escandallo!$D$10)*Datos!$B$11</f>
-        <v/>
+        <v>33922.02739726025</v>
       </c>
       <c r="I8" s="68">
         <f>Datos!$B$14*(I$4-(Escandallo!$D$6*(1+$A8)+Escandallo!$D$7+Escandallo!$D$8+Escandallo!$D$9))-Datos!$B$50-Datos!$B$53-(I$4*Datos!$B$14*Datos!$B$17/365+Datos!$B$18*Escandallo!$D$10)*Datos!$B$11</f>
-        <v/>
+        <v>77257.64383561641</v>
       </c>
     </row>
     <row r="9">
@@ -1198,35 +1198,35 @@
       </c>
       <c r="B9" s="68">
         <f>Datos!$B$14*(B$4-(Escandallo!$D$6*(1+$A9)+Escandallo!$D$7+Escandallo!$D$8+Escandallo!$D$9))-Datos!$B$50-Datos!$B$53-(B$4*Datos!$B$14*Datos!$B$17/365+Datos!$B$18*Escandallo!$D$10)*Datos!$B$11</f>
-        <v/>
+        <v>-263306.67123287666</v>
       </c>
       <c r="C9" s="68">
         <f>Datos!$B$14*(C$4-(Escandallo!$D$6*(1+$A9)+Escandallo!$D$7+Escandallo!$D$8+Escandallo!$D$9))-Datos!$B$50-Datos!$B$53-(C$4*Datos!$B$14*Datos!$B$17/365+Datos!$B$18*Escandallo!$D$10)*Datos!$B$11</f>
-        <v/>
+        <v>-219971.0547945205</v>
       </c>
       <c r="D9" s="68">
         <f>Datos!$B$14*(D$4-(Escandallo!$D$6*(1+$A9)+Escandallo!$D$7+Escandallo!$D$8+Escandallo!$D$9))-Datos!$B$50-Datos!$B$53-(D$4*Datos!$B$14*Datos!$B$17/365+Datos!$B$18*Escandallo!$D$10)*Datos!$B$11</f>
-        <v/>
+        <v>-176635.43835616432</v>
       </c>
       <c r="E9" s="68">
         <f>Datos!$B$14*(E$4-(Escandallo!$D$6*(1+$A9)+Escandallo!$D$7+Escandallo!$D$8+Escandallo!$D$9))-Datos!$B$50-Datos!$B$53-(E$4*Datos!$B$14*Datos!$B$17/365+Datos!$B$18*Escandallo!$D$10)*Datos!$B$11</f>
-        <v/>
+        <v>-133299.82191780818</v>
       </c>
       <c r="F9" s="68">
         <f>Datos!$B$14*(F$4-(Escandallo!$D$6*(1+$A9)+Escandallo!$D$7+Escandallo!$D$8+Escandallo!$D$9))-Datos!$B$50-Datos!$B$53-(F$4*Datos!$B$14*Datos!$B$17/365+Datos!$B$18*Escandallo!$D$10)*Datos!$B$11</f>
-        <v/>
+        <v>-89964.20547945201</v>
       </c>
       <c r="G9" s="68">
         <f>Datos!$B$14*(G$4-(Escandallo!$D$6*(1+$A9)+Escandallo!$D$7+Escandallo!$D$8+Escandallo!$D$9))-Datos!$B$50-Datos!$B$53-(G$4*Datos!$B$14*Datos!$B$17/365+Datos!$B$18*Escandallo!$D$10)*Datos!$B$11</f>
-        <v/>
+        <v>-46628.589041095845</v>
       </c>
       <c r="H9" s="68">
         <f>Datos!$B$14*(H$4-(Escandallo!$D$6*(1+$A9)+Escandallo!$D$7+Escandallo!$D$8+Escandallo!$D$9))-Datos!$B$50-Datos!$B$53-(H$4*Datos!$B$14*Datos!$B$17/365+Datos!$B$18*Escandallo!$D$10)*Datos!$B$11</f>
-        <v/>
+        <v>-3292.97260273969</v>
       </c>
       <c r="I9" s="68">
         <f>Datos!$B$14*(I$4-(Escandallo!$D$6*(1+$A9)+Escandallo!$D$7+Escandallo!$D$8+Escandallo!$D$9))-Datos!$B$50-Datos!$B$53-(I$4*Datos!$B$14*Datos!$B$17/365+Datos!$B$18*Escandallo!$D$10)*Datos!$B$11</f>
-        <v/>
+        <v>40042.64383561647</v>
       </c>
     </row>
     <row r="10">
@@ -1235,35 +1235,35 @@
       </c>
       <c r="B10" s="68">
         <f>Datos!$B$14*(B$4-(Escandallo!$D$6*(1+$A10)+Escandallo!$D$7+Escandallo!$D$8+Escandallo!$D$9))-Datos!$B$50-Datos!$B$53-(B$4*Datos!$B$14*Datos!$B$17/365+Datos!$B$18*Escandallo!$D$10)*Datos!$B$11</f>
-        <v/>
+        <v>-300521.6712328766</v>
       </c>
       <c r="C10" s="68">
         <f>Datos!$B$14*(C$4-(Escandallo!$D$6*(1+$A10)+Escandallo!$D$7+Escandallo!$D$8+Escandallo!$D$9))-Datos!$B$50-Datos!$B$53-(C$4*Datos!$B$14*Datos!$B$17/365+Datos!$B$18*Escandallo!$D$10)*Datos!$B$11</f>
-        <v/>
+        <v>-257186.05479452043</v>
       </c>
       <c r="D10" s="68">
         <f>Datos!$B$14*(D$4-(Escandallo!$D$6*(1+$A10)+Escandallo!$D$7+Escandallo!$D$8+Escandallo!$D$9))-Datos!$B$50-Datos!$B$53-(D$4*Datos!$B$14*Datos!$B$17/365+Datos!$B$18*Escandallo!$D$10)*Datos!$B$11</f>
-        <v/>
+        <v>-213850.43835616426</v>
       </c>
       <c r="E10" s="68">
         <f>Datos!$B$14*(E$4-(Escandallo!$D$6*(1+$A10)+Escandallo!$D$7+Escandallo!$D$8+Escandallo!$D$9))-Datos!$B$50-Datos!$B$53-(E$4*Datos!$B$14*Datos!$B$17/365+Datos!$B$18*Escandallo!$D$10)*Datos!$B$11</f>
-        <v/>
+        <v>-170514.8219178081</v>
       </c>
       <c r="F10" s="68">
         <f>Datos!$B$14*(F$4-(Escandallo!$D$6*(1+$A10)+Escandallo!$D$7+Escandallo!$D$8+Escandallo!$D$9))-Datos!$B$50-Datos!$B$53-(F$4*Datos!$B$14*Datos!$B$17/365+Datos!$B$18*Escandallo!$D$10)*Datos!$B$11</f>
-        <v/>
+        <v>-127179.20547945194</v>
       </c>
       <c r="G10" s="68">
         <f>Datos!$B$14*(G$4-(Escandallo!$D$6*(1+$A10)+Escandallo!$D$7+Escandallo!$D$8+Escandallo!$D$9))-Datos!$B$50-Datos!$B$53-(G$4*Datos!$B$14*Datos!$B$17/365+Datos!$B$18*Escandallo!$D$10)*Datos!$B$11</f>
-        <v/>
+        <v>-83843.58904109575</v>
       </c>
       <c r="H10" s="68">
         <f>Datos!$B$14*(H$4-(Escandallo!$D$6*(1+$A10)+Escandallo!$D$7+Escandallo!$D$8+Escandallo!$D$9))-Datos!$B$50-Datos!$B$53-(H$4*Datos!$B$14*Datos!$B$17/365+Datos!$B$18*Escandallo!$D$10)*Datos!$B$11</f>
-        <v/>
+        <v>-40507.97260273959</v>
       </c>
       <c r="I10" s="68">
         <f>Datos!$B$14*(I$4-(Escandallo!$D$6*(1+$A10)+Escandallo!$D$7+Escandallo!$D$8+Escandallo!$D$9))-Datos!$B$50-Datos!$B$53-(I$4*Datos!$B$14*Datos!$B$17/365+Datos!$B$18*Escandallo!$D$10)*Datos!$B$11</f>
-        <v/>
+        <v>2827.64383561656</v>
       </c>
     </row>
     <row r="11">
@@ -1272,35 +1272,35 @@
       </c>
       <c r="B11" s="68">
         <f>Datos!$B$14*(B$4-(Escandallo!$D$6*(1+$A11)+Escandallo!$D$7+Escandallo!$D$8+Escandallo!$D$9))-Datos!$B$50-Datos!$B$53-(B$4*Datos!$B$14*Datos!$B$17/365+Datos!$B$18*Escandallo!$D$10)*Datos!$B$11</f>
-        <v/>
+        <v>-337736.67123287666</v>
       </c>
       <c r="C11" s="68">
         <f>Datos!$B$14*(C$4-(Escandallo!$D$6*(1+$A11)+Escandallo!$D$7+Escandallo!$D$8+Escandallo!$D$9))-Datos!$B$50-Datos!$B$53-(C$4*Datos!$B$14*Datos!$B$17/365+Datos!$B$18*Escandallo!$D$10)*Datos!$B$11</f>
-        <v/>
+        <v>-294401.0547945205</v>
       </c>
       <c r="D11" s="68">
         <f>Datos!$B$14*(D$4-(Escandallo!$D$6*(1+$A11)+Escandallo!$D$7+Escandallo!$D$8+Escandallo!$D$9))-Datos!$B$50-Datos!$B$53-(D$4*Datos!$B$14*Datos!$B$17/365+Datos!$B$18*Escandallo!$D$10)*Datos!$B$11</f>
-        <v/>
+        <v>-251065.43835616432</v>
       </c>
       <c r="E11" s="68">
         <f>Datos!$B$14*(E$4-(Escandallo!$D$6*(1+$A11)+Escandallo!$D$7+Escandallo!$D$8+Escandallo!$D$9))-Datos!$B$50-Datos!$B$53-(E$4*Datos!$B$14*Datos!$B$17/365+Datos!$B$18*Escandallo!$D$10)*Datos!$B$11</f>
-        <v/>
+        <v>-207729.82191780815</v>
       </c>
       <c r="F11" s="68">
         <f>Datos!$B$14*(F$4-(Escandallo!$D$6*(1+$A11)+Escandallo!$D$7+Escandallo!$D$8+Escandallo!$D$9))-Datos!$B$50-Datos!$B$53-(F$4*Datos!$B$14*Datos!$B$17/365+Datos!$B$18*Escandallo!$D$10)*Datos!$B$11</f>
-        <v/>
+        <v>-164394.205479452</v>
       </c>
       <c r="G11" s="68">
         <f>Datos!$B$14*(G$4-(Escandallo!$D$6*(1+$A11)+Escandallo!$D$7+Escandallo!$D$8+Escandallo!$D$9))-Datos!$B$50-Datos!$B$53-(G$4*Datos!$B$14*Datos!$B$17/365+Datos!$B$18*Escandallo!$D$10)*Datos!$B$11</f>
-        <v/>
+        <v>-121058.58904109584</v>
       </c>
       <c r="H11" s="68">
         <f>Datos!$B$14*(H$4-(Escandallo!$D$6*(1+$A11)+Escandallo!$D$7+Escandallo!$D$8+Escandallo!$D$9))-Datos!$B$50-Datos!$B$53-(H$4*Datos!$B$14*Datos!$B$17/365+Datos!$B$18*Escandallo!$D$10)*Datos!$B$11</f>
-        <v/>
+        <v>-77722.97260273967</v>
       </c>
       <c r="I11" s="68">
         <f>Datos!$B$14*(I$4-(Escandallo!$D$6*(1+$A11)+Escandallo!$D$7+Escandallo!$D$8+Escandallo!$D$9))-Datos!$B$50-Datos!$B$53-(I$4*Datos!$B$14*Datos!$B$17/365+Datos!$B$18*Escandallo!$D$10)*Datos!$B$11</f>
-        <v/>
+        <v>-34387.35616438351</v>
       </c>
     </row>
     <row r="13">
@@ -1363,15 +1363,15 @@
       </c>
       <c r="B19" s="18">
         <f>Datos!$B$14*Datos!$B$15*A19/365+Datos!$B$18*Escandallo!$D$10</f>
-        <v/>
+        <v>84492.60273972603</v>
       </c>
       <c r="C19" s="18">
         <f>-B19*Datos!$B$11</f>
-        <v/>
+        <v>-6336.945205479452</v>
       </c>
       <c r="D19" s="38">
         <f>Persan!$B$7-Datos!$B$50-Datos!$B$53+C19</f>
-        <v/>
+        <v>-161136.94520547945</v>
       </c>
     </row>
     <row r="20">
@@ -1380,15 +1380,15 @@
       </c>
       <c r="B20" s="18">
         <f>Datos!$B$14*Datos!$B$15*A20/365+Datos!$B$18*Escandallo!$D$10</f>
-        <v/>
+        <v>158465.20547945207</v>
       </c>
       <c r="C20" s="18">
         <f>-B20*Datos!$B$11</f>
-        <v/>
+        <v>-11884.890410958904</v>
       </c>
       <c r="D20" s="38">
         <f>Persan!$B$7-Datos!$B$50-Datos!$B$53+C20</f>
-        <v/>
+        <v>-166684.8904109589</v>
       </c>
     </row>
     <row r="21">
@@ -1397,15 +1397,15 @@
       </c>
       <c r="B21" s="18">
         <f>Datos!$B$14*Datos!$B$15*A21/365+Datos!$B$18*Escandallo!$D$10</f>
-        <v/>
+        <v>232437.80821917808</v>
       </c>
       <c r="C21" s="18">
         <f>-B21*Datos!$B$11</f>
-        <v/>
+        <v>-17432.835616438355</v>
       </c>
       <c r="D21" s="38">
         <f>Persan!$B$7-Datos!$B$50-Datos!$B$53+C21</f>
-        <v/>
+        <v>-172232.83561643836</v>
       </c>
     </row>
     <row r="22">
@@ -1414,15 +1414,15 @@
       </c>
       <c r="B22" s="18">
         <f>Datos!$B$14*Datos!$B$15*A22/365+Datos!$B$18*Escandallo!$D$10</f>
-        <v/>
+        <v>306410.41095890413</v>
       </c>
       <c r="C22" s="18">
         <f>-B22*Datos!$B$11</f>
-        <v/>
+        <v>-22980.780821917808</v>
       </c>
       <c r="D22" s="38">
         <f>Persan!$B$7-Datos!$B$50-Datos!$B$53+C22</f>
-        <v/>
+        <v>-177780.7808219178</v>
       </c>
     </row>
     <row r="23">
@@ -1431,15 +1431,15 @@
       </c>
       <c r="B23" s="18">
         <f>Datos!$B$14*Datos!$B$15*A23/365+Datos!$B$18*Escandallo!$D$10</f>
-        <v/>
+        <v>454355.61643835617</v>
       </c>
       <c r="C23" s="18">
         <f>-B23*Datos!$B$11</f>
-        <v/>
+        <v>-34076.67123287671</v>
       </c>
       <c r="D23" s="38">
         <f>Persan!$B$7-Datos!$B$50-Datos!$B$53+C23</f>
-        <v/>
+        <v>-188876.67123287672</v>
       </c>
     </row>
     <row r="24">
@@ -1529,7 +1529,7 @@
       </c>
       <c r="B7" s="14">
         <f>Datos!$B$5*Datos!$B$6</f>
-        <v/>
+        <v>242.0</v>
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
@@ -1753,7 +1753,7 @@
       </c>
       <c r="B26" s="18">
         <f>Datos!$B$24/Datos!$B$25</f>
-        <v/>
+        <v>36000.0</v>
       </c>
       <c r="C26" s="9" t="inlineStr">
         <is>
@@ -1823,7 +1823,7 @@
       </c>
       <c r="B33" s="20">
         <f>Datos!$B$32/Datos!$B$31</f>
-        <v/>
+        <v>62.5</v>
       </c>
       <c r="C33" s="9" t="inlineStr">
         <is>
@@ -1883,7 +1883,7 @@
       </c>
       <c r="B39" s="14">
         <f>Datos!$B$38*12</f>
-        <v/>
+        <v>360000.0</v>
       </c>
     </row>
     <row r="41">
@@ -1992,7 +1992,7 @@
       </c>
       <c r="B50" s="18">
         <f>Datos!$B$49*12</f>
-        <v/>
+        <v>60000.0</v>
       </c>
     </row>
     <row r="51">
@@ -2033,7 +2033,7 @@
       </c>
       <c r="B53" s="18">
         <f>Datos!$B$52*12</f>
-        <v/>
+        <v>48000.0</v>
       </c>
     </row>
     <row r="54">
@@ -2054,7 +2054,7 @@
       </c>
       <c r="B55" s="18">
         <f>Datos!$B$42+Datos!$B$51</f>
-        <v/>
+        <v>190000.0</v>
       </c>
       <c r="C55" s="9" t="inlineStr">
         <is>
@@ -2232,7 +2232,7 @@
       </c>
       <c r="C5" s="28">
         <f>B5/$B$5</f>
-        <v/>
+        <v>1.0</v>
       </c>
       <c r="D5" s="29" t="n"/>
       <c r="E5" s="29" t="n"/>
@@ -2248,7 +2248,7 @@
       </c>
       <c r="C6" s="30">
         <f>B6/$B$5</f>
-        <v/>
+        <v>0.08201528940408487</v>
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
@@ -2267,7 +2267,7 @@
       </c>
       <c r="C7" s="30">
         <f>B7/$B$5</f>
-        <v/>
+        <v>-0.6692098846152252</v>
       </c>
       <c r="F7" s="9" t="inlineStr">
         <is>
@@ -2283,18 +2283,18 @@
       </c>
       <c r="B8" s="27">
         <f>SUM(B5:B7)</f>
-        <v/>
+        <v>1892823.0</v>
       </c>
       <c r="C8" s="28">
         <f>B8/$B$5</f>
-        <v/>
+        <v>0.41280540478885963</v>
       </c>
       <c r="D8" s="31" t="n">
         <v>1892822</v>
       </c>
       <c r="E8" s="32">
         <f>B8-D8</f>
-        <v/>
+        <v>1.0</v>
       </c>
     </row>
     <row r="9">
@@ -2308,7 +2308,7 @@
       </c>
       <c r="C9" s="30">
         <f>B9/$B$5</f>
-        <v/>
+        <v>-0.10504513695712812</v>
       </c>
     </row>
     <row r="10">
@@ -2322,7 +2322,7 @@
       </c>
       <c r="C10" s="30">
         <f>B10/$B$5</f>
-        <v/>
+        <v>-0.05849561214210645</v>
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
@@ -2341,7 +2341,7 @@
       </c>
       <c r="C11" s="30">
         <f>B11/$B$5</f>
-        <v/>
+        <v>-0.06788961253510428</v>
       </c>
     </row>
     <row r="12">
@@ -2355,7 +2355,7 @@
       </c>
       <c r="C12" s="30">
         <f>B12/$B$5</f>
-        <v/>
+        <v>-0.08265145737423797</v>
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
@@ -2371,18 +2371,18 @@
       </c>
       <c r="B13" s="27">
         <f>B8+SUM(B9:B12)</f>
-        <v/>
+        <v>452674.0</v>
       </c>
       <c r="C13" s="28">
         <f>B13/$B$5</f>
-        <v/>
+        <v>0.0987235857802828</v>
       </c>
       <c r="D13" s="31" t="n">
         <v>452674</v>
       </c>
       <c r="E13" s="32">
         <f>B13-D13</f>
-        <v/>
+        <v>0.0</v>
       </c>
     </row>
     <row r="14">
@@ -2396,7 +2396,7 @@
       </c>
       <c r="C14" s="30">
         <f>B14/$B$5</f>
-        <v/>
+        <v>-0.007882419933233987</v>
       </c>
       <c r="F14" s="9" t="inlineStr">
         <is>
@@ -2412,18 +2412,18 @@
       </c>
       <c r="B15" s="27">
         <f>B13+B14</f>
-        <v/>
+        <v>416531.0</v>
       </c>
       <c r="C15" s="28">
         <f>B15/$B$5</f>
-        <v/>
+        <v>0.09084116584704882</v>
       </c>
       <c r="D15" s="31" t="n">
         <v>416531</v>
       </c>
       <c r="E15" s="32">
         <f>B15-D15</f>
-        <v/>
+        <v>0.0</v>
       </c>
     </row>
     <row r="16">
@@ -2437,7 +2437,7 @@
       </c>
       <c r="C16" s="30">
         <f>B16/$B$5</f>
-        <v/>
+        <v>-0.009605983686446176</v>
       </c>
     </row>
     <row r="17">
@@ -2448,18 +2448,18 @@
       </c>
       <c r="B17" s="27">
         <f>B15+B16</f>
-        <v/>
+        <v>372485.0</v>
       </c>
       <c r="C17" s="28">
         <f>B17/$B$5</f>
-        <v/>
+        <v>0.08123518216060265</v>
       </c>
       <c r="D17" s="31" t="n">
         <v>372485</v>
       </c>
       <c r="E17" s="32">
         <f>B17-D17</f>
-        <v/>
+        <v>0.0</v>
       </c>
     </row>
     <row r="18">
@@ -2473,7 +2473,7 @@
       </c>
       <c r="C18" s="30">
         <f>B18/$B$5</f>
-        <v/>
+        <v>-0.020308741017698643</v>
       </c>
     </row>
     <row r="19">
@@ -2484,18 +2484,18 @@
       </c>
       <c r="B19" s="27">
         <f>B17+B18</f>
-        <v/>
+        <v>279364.0</v>
       </c>
       <c r="C19" s="28">
         <f>B19/$B$5</f>
-        <v/>
+        <v>0.060926441142904</v>
       </c>
       <c r="D19" s="31" t="n">
         <v>279364</v>
       </c>
       <c r="E19" s="32">
         <f>B19-D19</f>
-        <v/>
+        <v>0.0</v>
       </c>
     </row>
     <row r="21">
@@ -2518,7 +2518,7 @@
       </c>
       <c r="B22" s="30">
         <f>PyG2025!$B$18/-PyG2025!$B$17</f>
-        <v/>
+        <v>0.24999932883203352</v>
       </c>
       <c r="C22" s="9" t="inlineStr">
         <is>
@@ -2534,7 +2534,7 @@
       </c>
       <c r="B23" s="30">
         <f>PyG2025!$B$13/PyG2025!$B$5</f>
-        <v/>
+        <v>0.0987235857802828</v>
       </c>
     </row>
     <row r="24">
@@ -2545,7 +2545,7 @@
       </c>
       <c r="B24" s="30">
         <f>PyG2025!$B$19/PyG2025!$B$5</f>
-        <v/>
+        <v>0.060926441142904</v>
       </c>
     </row>
     <row r="26">
@@ -2568,7 +2568,7 @@
       </c>
       <c r="B27" s="33">
         <f>PyG2025!$B$13</f>
-        <v/>
+        <v>452674.0</v>
       </c>
     </row>
     <row r="28">
@@ -2579,7 +2579,7 @@
       </c>
       <c r="B28" s="33">
         <f>-PyG2025!$B$6</f>
-        <v/>
+        <v>-376062.0</v>
       </c>
       <c r="C28" s="9" t="inlineStr">
         <is>
@@ -2595,7 +2595,7 @@
       </c>
       <c r="B29" s="33">
         <f>PyG2025!$B$16</f>
-        <v/>
+        <v>-44046.0</v>
       </c>
     </row>
     <row r="30">
@@ -2606,7 +2606,7 @@
       </c>
       <c r="B30" s="33">
         <f>PyG2025!$B$18</f>
-        <v/>
+        <v>-93121.0</v>
       </c>
     </row>
     <row r="31">
@@ -2617,7 +2617,7 @@
       </c>
       <c r="B31" s="35">
         <f>B27+B28+B29+B30</f>
-        <v/>
+        <v>-60555.0</v>
       </c>
       <c r="C31" s="36" t="n"/>
       <c r="D31" s="36" t="n"/>
@@ -2717,15 +2717,15 @@
       </c>
       <c r="D5" s="38">
         <f>B5+C5</f>
-        <v/>
+        <v>4585266.0</v>
       </c>
       <c r="E5" s="33">
         <f>PyG2025!$B$5</f>
-        <v/>
+        <v>4585267.0</v>
       </c>
       <c r="F5" s="18">
         <f>D5-E5</f>
-        <v/>
+        <v>-1.0</v>
       </c>
     </row>
     <row r="6">
@@ -2742,15 +2742,15 @@
       </c>
       <c r="D6" s="38">
         <f>B6+C6</f>
-        <v/>
+        <v>279364.0</v>
       </c>
       <c r="E6" s="33">
         <f>PyG2025!$B$19</f>
-        <v/>
+        <v>279364.0</v>
       </c>
       <c r="F6" s="18">
         <f>D6-E6</f>
-        <v/>
+        <v>0.0</v>
       </c>
     </row>
     <row r="7">
@@ -2767,7 +2767,7 @@
       </c>
       <c r="D7" s="39">
         <f>B7+C7</f>
-        <v/>
+        <v>434834.0</v>
       </c>
     </row>
     <row r="9">
@@ -2790,11 +2790,11 @@
       </c>
       <c r="B10" s="40">
         <f>B5/B7</f>
-        <v/>
+        <v>15.158529317379545</v>
       </c>
       <c r="C10" s="40">
         <f>C5/C7</f>
-        <v/>
+        <v>7.452241385933238</v>
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
@@ -2810,11 +2810,11 @@
       </c>
       <c r="B11" s="40">
         <f>B6/B7</f>
-        <v/>
+        <v>0.9104776967863201</v>
       </c>
       <c r="C11" s="40">
         <f>C6/C7</f>
-        <v/>
+        <v>0.4628049014712096</v>
       </c>
     </row>
     <row r="12">
@@ -2825,11 +2825,11 @@
       </c>
       <c r="B12" s="30">
         <f>B6/B5</f>
-        <v/>
+        <v>0.060063722391752075</v>
       </c>
       <c r="C12" s="30">
         <f>C6/C5</f>
-        <v/>
+        <v>0.06210277921818187</v>
       </c>
     </row>
     <row r="13">
@@ -2840,11 +2840,11 @@
       </c>
       <c r="B13" s="30">
         <f>B5/$D$5</f>
-        <v/>
+        <v>0.5768965202891173</v>
       </c>
       <c r="C13" s="30">
         <f>C5/$D$5</f>
-        <v/>
+        <v>0.42310347971088264</v>
       </c>
     </row>
     <row r="14">
@@ -2855,11 +2855,11 @@
       </c>
       <c r="B14" s="30">
         <f>B6/$D$6</f>
-        <v/>
+        <v>0.5687275382654887</v>
       </c>
       <c r="C14" s="30">
         <f>C6/$D$6</f>
-        <v/>
+        <v>0.4312724617345112</v>
       </c>
       <c r="F14" s="9" t="inlineStr">
         <is>
@@ -3044,15 +3044,15 @@
       </c>
       <c r="B10" s="41">
         <f>SUM(B6:B9)</f>
-        <v/>
+        <v>12.37</v>
       </c>
       <c r="C10" s="41">
         <f>SUM(C6:C9)</f>
-        <v/>
+        <v>7.0200000000000005</v>
       </c>
       <c r="D10" s="41">
         <f>SUM(D6:D9)</f>
-        <v/>
+        <v>10.52</v>
       </c>
       <c r="E10" s="29" t="n"/>
       <c r="F10" s="42" t="inlineStr">
@@ -3069,15 +3069,15 @@
       </c>
       <c r="B11" s="41">
         <f>B5-B10</f>
-        <v/>
+        <v>2.790000000000001</v>
       </c>
       <c r="C11" s="41">
         <f>C5-C10</f>
-        <v/>
+        <v>0.4299999999999997</v>
       </c>
       <c r="D11" s="43">
         <f>D5-D10</f>
-        <v/>
+        <v>-0.5199999999999996</v>
       </c>
       <c r="F11" s="44" t="inlineStr">
         <is>
@@ -3093,15 +3093,15 @@
       </c>
       <c r="B12" s="30">
         <f>B11/B5</f>
-        <v/>
+        <v>0.18403693931398424</v>
       </c>
       <c r="C12" s="30">
         <f>C11/C5</f>
-        <v/>
+        <v>0.05771812080536909</v>
       </c>
       <c r="D12" s="30">
         <f>D11/D5</f>
-        <v/>
+        <v>-0.051999999999999956</v>
       </c>
     </row>
     <row r="13">
@@ -3112,15 +3112,15 @@
       </c>
       <c r="B13" s="30">
         <f>B6/B5</f>
-        <v/>
+        <v>0.5455145118733509</v>
       </c>
       <c r="C13" s="30">
         <f>C6/C5</f>
-        <v/>
+        <v>0.6442953020134228</v>
       </c>
       <c r="D13" s="30">
         <f>D6/D5</f>
-        <v/>
+        <v>0.827</v>
       </c>
       <c r="F13" s="9" t="inlineStr">
         <is>
@@ -3180,19 +3180,19 @@
       </c>
       <c r="B17" s="18">
         <f>Escandallo!$B$6*Lineas!$B$7+Escandallo!$C$6*Lineas!$C$7</f>
-        <v/>
+        <v>2692732.08</v>
       </c>
       <c r="C17" s="33">
         <f>-(PyG2025!$B$7+PyG2025!$B$6)</f>
-        <v/>
+        <v>2692444.0</v>
       </c>
       <c r="D17" s="18">
         <f>B17-C17</f>
-        <v/>
+        <v>288.0800000000745</v>
       </c>
       <c r="E17" s="30">
         <f>IF(C17=0,0,(B17-C17)/C17)</f>
-        <v/>
+        <v>0.00010699572581642349</v>
       </c>
       <c r="F17" s="9" t="inlineStr">
         <is>
@@ -3208,19 +3208,19 @@
       </c>
       <c r="B18" s="18">
         <f>Escandallo!$B$8*Lineas!$B$7+Escandallo!$C$8*Lineas!$C$7</f>
-        <v/>
+        <v>269597.08</v>
       </c>
       <c r="C18" s="33">
         <f>-PyG2025!$B$10</f>
-        <v/>
+        <v>268218.0</v>
       </c>
       <c r="D18" s="18">
         <f>B18-C18</f>
-        <v/>
+        <v>1379.0800000000163</v>
       </c>
       <c r="E18" s="30">
         <f>IF(C18=0,0,(B18-C18)/C18)</f>
-        <v/>
+        <v>0.0051416385179220495</v>
       </c>
       <c r="F18" s="9" t="inlineStr">
         <is>
@@ -3236,19 +3236,19 @@
       </c>
       <c r="B19" s="18">
         <f>Escandallo!$B$9*Lineas!$B$7+Escandallo!$C$9*Lineas!$C$7</f>
-        <v/>
+        <v>377846.6</v>
       </c>
       <c r="C19" s="33">
         <f>-PyG2025!$B$12</f>
-        <v/>
+        <v>378979.0</v>
       </c>
       <c r="D19" s="18">
         <f>B19-C19</f>
-        <v/>
+        <v>-1132.4000000000233</v>
       </c>
       <c r="E19" s="30">
         <f>IF(C19=0,0,(B19-C19)/C19)</f>
-        <v/>
+        <v>-0.002988028360410533</v>
       </c>
       <c r="F19" s="9" t="inlineStr">
         <is>
@@ -3264,19 +3264,19 @@
       </c>
       <c r="B20" s="18">
         <f>Escandallo!$B$7*Lineas!$B$7+Escandallo!$C$7*Lineas!$C$7</f>
-        <v/>
+        <v>645955.3200000001</v>
       </c>
       <c r="C20" s="33">
         <f>-PyG2025!$B$9</f>
-        <v/>
+        <v>481660.0</v>
       </c>
       <c r="D20" s="18">
         <f>B20-C20</f>
-        <v/>
+        <v>164295.32000000007</v>
       </c>
       <c r="E20" s="30">
         <f>IF(C20=0,0,(B20-C20)/C20)</f>
-        <v/>
+        <v>0.3411022713117138</v>
       </c>
       <c r="F20" s="9" t="inlineStr">
         <is>
@@ -3304,7 +3304,7 @@
       </c>
       <c r="B23" s="20">
         <f>Escandallo!$B$7*Lineas!$B$7/Datos!$B$9</f>
-        <v/>
+        <v>10.011018947368422</v>
       </c>
       <c r="F23" s="9" t="inlineStr">
         <is>
@@ -3320,7 +3320,7 @@
       </c>
       <c r="B24" s="20">
         <f>Escandallo!$C$7*Lineas!$C$7/Datos!$B$9</f>
-        <v/>
+        <v>6.987805263157894</v>
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
@@ -3416,19 +3416,19 @@
       </c>
       <c r="B6" s="14">
         <f>Datos!$B$21*Datos!$B$22*Datos!$B$8</f>
-        <v/>
+        <v>390.0</v>
       </c>
       <c r="C6" s="45">
         <f>Datos!$B$7</f>
-        <v/>
+        <v>242.0</v>
       </c>
       <c r="D6" s="14">
         <f>B6*C6</f>
-        <v/>
+        <v>94380.0</v>
       </c>
       <c r="E6" s="45">
         <f>Datos!$B$23</f>
-        <v/>
+        <v>2.0</v>
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
@@ -3444,19 +3444,19 @@
       </c>
       <c r="B7" s="45">
         <f>Datos!$B$32</f>
-        <v/>
+        <v>500.0</v>
       </c>
       <c r="C7" s="45">
         <f>Datos!$B$7</f>
-        <v/>
+        <v>242.0</v>
       </c>
       <c r="D7" s="14">
         <f>B7*C7</f>
-        <v/>
+        <v>121000.0</v>
       </c>
       <c r="E7" s="45">
         <f>Datos!$B$31</f>
-        <v/>
+        <v>8.0</v>
       </c>
       <c r="F7" s="9" t="inlineStr">
         <is>
@@ -3472,16 +3472,16 @@
       </c>
       <c r="B8" s="46">
         <f>B6+B7</f>
-        <v/>
+        <v>890.0</v>
       </c>
       <c r="C8" s="29" t="n"/>
       <c r="D8" s="46">
         <f>D6+D7</f>
-        <v/>
+        <v>215380.0</v>
       </c>
       <c r="E8" s="46">
         <f>E6+E7</f>
-        <v/>
+        <v>10.0</v>
       </c>
       <c r="F8" s="29" t="n"/>
     </row>
@@ -3505,7 +3505,7 @@
       </c>
       <c r="B11" s="45">
         <f>Lineas!$B$7</f>
-        <v/>
+        <v>174504.0</v>
       </c>
     </row>
     <row r="12">
@@ -3516,7 +3516,7 @@
       </c>
       <c r="B12" s="45">
         <f>Capacidad!$D$8</f>
-        <v/>
+        <v>215380.0</v>
       </c>
     </row>
     <row r="13">
@@ -3527,7 +3527,7 @@
       </c>
       <c r="B13" s="47">
         <f>B11/B12</f>
-        <v/>
+        <v>0.8102145045965271</v>
       </c>
       <c r="F13" s="9" t="inlineStr">
         <is>
@@ -3543,7 +3543,7 @@
       </c>
       <c r="B14" s="39">
         <f>B12-B11</f>
-        <v/>
+        <v>40876.0</v>
       </c>
       <c r="F14" s="9" t="inlineStr">
         <is>
@@ -3571,7 +3571,7 @@
       </c>
       <c r="B17" s="14">
         <f>Datos!$B$43*Datos!$B$44</f>
-        <v/>
+        <v>360.0</v>
       </c>
       <c r="F17" s="9" t="inlineStr">
         <is>
@@ -3587,7 +3587,7 @@
       </c>
       <c r="B18" s="39">
         <f>B17*Datos!$B$7</f>
-        <v/>
+        <v>87120.0</v>
       </c>
     </row>
     <row r="19">
@@ -3598,7 +3598,7 @@
       </c>
       <c r="B19" s="20">
         <f>Datos!$B$14/Datos!$B$7</f>
-        <v/>
+        <v>371.900826446281</v>
       </c>
       <c r="F19" s="9" t="inlineStr">
         <is>
@@ -3614,7 +3614,7 @@
       </c>
       <c r="B20" s="45">
         <f>Datos!$B$14</f>
-        <v/>
+        <v>90000.0</v>
       </c>
     </row>
     <row r="21">
@@ -3625,7 +3625,7 @@
       </c>
       <c r="B21" s="48">
         <f>B18-B20</f>
-        <v/>
+        <v>-2880.0</v>
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
@@ -3641,7 +3641,7 @@
       </c>
       <c r="B22" s="30">
         <f>B21/B20</f>
-        <v/>
+        <v>-0.032</v>
       </c>
     </row>
     <row r="24">
@@ -3696,19 +3696,19 @@
       </c>
       <c r="B26" s="14">
         <f>Capacidad!$D$8</f>
-        <v/>
+        <v>215380.0</v>
       </c>
       <c r="C26" s="14">
         <f>Lineas!$B$7</f>
-        <v/>
+        <v>174504.0</v>
       </c>
       <c r="D26" s="39">
         <f>B26-C26</f>
-        <v/>
-      </c>
-      <c r="E26" s="49">
+        <v>40876.0</v>
+      </c>
+      <c t="str" r="E26" s="49">
         <f>IF(D26&gt;=0,"SÍ","NO")</f>
-        <v/>
+        <v>SÍ</v>
       </c>
       <c r="F26" s="9" t="inlineStr">
         <is>
@@ -3724,19 +3724,19 @@
       </c>
       <c r="B27" s="14">
         <f>Capacidad!$D$8</f>
-        <v/>
+        <v>215380.0</v>
       </c>
       <c r="C27" s="14">
         <f>Lineas!$B$7+Datos!$B$14</f>
-        <v/>
+        <v>264504.0</v>
       </c>
       <c r="D27" s="39">
         <f>B27-C27</f>
-        <v/>
-      </c>
-      <c r="E27" s="49">
+        <v>-49124.0</v>
+      </c>
+      <c t="str" r="E27" s="49">
         <f>IF(D27&gt;=0,"SÍ","NO")</f>
-        <v/>
+        <v>NO</v>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
@@ -3752,19 +3752,19 @@
       </c>
       <c r="B28" s="14">
         <f>Capacidad!$D$8+Capacidad!$B$18</f>
-        <v/>
+        <v>302500.0</v>
       </c>
       <c r="C28" s="14">
         <f>Lineas!$B$7+Datos!$B$14</f>
-        <v/>
+        <v>264504.0</v>
       </c>
       <c r="D28" s="39">
         <f>B28-C28</f>
-        <v/>
-      </c>
-      <c r="E28" s="49">
+        <v>37996.0</v>
+      </c>
+      <c t="str" r="E28" s="49">
         <f>IF(D28&gt;=0,"SÍ","NO")</f>
-        <v/>
+        <v>SÍ</v>
       </c>
       <c r="F28" s="9" t="inlineStr">
         <is>
@@ -3780,19 +3780,19 @@
       </c>
       <c r="B29" s="14">
         <f>Capacidad!$D$8+Capacidad!$B$18</f>
-        <v/>
+        <v>302500.0</v>
       </c>
       <c r="C29" s="14">
         <f>Lineas!$B$7</f>
-        <v/>
+        <v>174504.0</v>
       </c>
       <c r="D29" s="39">
         <f>B29-C29</f>
-        <v/>
-      </c>
-      <c r="E29" s="49">
+        <v>127996.0</v>
+      </c>
+      <c t="str" r="E29" s="49">
         <f>IF(D29&gt;=0,"SÍ","NO")</f>
-        <v/>
+        <v>SÍ</v>
       </c>
       <c r="F29" s="9" t="inlineStr">
         <is>
@@ -3820,7 +3820,7 @@
       </c>
       <c r="B32" s="45">
         <f>Lineas!$C$7</f>
-        <v/>
+        <v>260330.0</v>
       </c>
     </row>
     <row r="33">
@@ -3831,7 +3831,7 @@
       </c>
       <c r="B33" s="14">
         <f>B32/12</f>
-        <v/>
+        <v>21694.166666666668</v>
       </c>
     </row>
     <row r="34">
@@ -3842,7 +3842,7 @@
       </c>
       <c r="B34" s="45">
         <f>Datos!$B$39</f>
-        <v/>
+        <v>360000.0</v>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
@@ -3858,7 +3858,7 @@
       </c>
       <c r="B35" s="39">
         <f>B34-B32</f>
-        <v/>
+        <v>99670.0</v>
       </c>
     </row>
     <row r="36">
@@ -3869,7 +3869,7 @@
       </c>
       <c r="B36" s="38">
         <f>B35*Escandallo!$C$11</f>
-        <v/>
+        <v>42858.09999999997</v>
       </c>
       <c r="F36" s="9" t="inlineStr">
         <is>
@@ -3885,7 +3885,7 @@
       </c>
       <c r="B37" s="20">
         <f>Datos!$B$39/(Datos!$B$7*Datos!$B$37)</f>
-        <v/>
+        <v>9.59744068248467</v>
       </c>
     </row>
     <row r="38">
@@ -3896,7 +3896,7 @@
       </c>
       <c r="B38" s="50">
         <f>B37-Datos!$B$36</f>
-        <v/>
+        <v>2.5974406824846703</v>
       </c>
       <c r="F38" s="9" t="inlineStr">
         <is>
@@ -3960,7 +3960,7 @@
       </c>
       <c r="B5" s="18">
         <f>Datos!$B$14*Datos!$B$15</f>
-        <v/>
+        <v>900000.0</v>
       </c>
     </row>
     <row r="6">
@@ -3971,7 +3971,7 @@
       </c>
       <c r="B6" s="18">
         <f>-Datos!$B$14*Escandallo!$D$10</f>
-        <v/>
+        <v>-946800.0</v>
       </c>
     </row>
     <row r="7">
@@ -3982,7 +3982,7 @@
       </c>
       <c r="B7" s="27">
         <f>B5+B6</f>
-        <v/>
+        <v>-46800.0</v>
       </c>
       <c r="C7" s="29" t="n"/>
       <c r="D7" s="29" t="n"/>
@@ -4001,7 +4001,7 @@
       </c>
       <c r="B8" s="33">
         <f>-Datos!$B$50</f>
-        <v/>
+        <v>-60000.0</v>
       </c>
       <c r="F8" s="9" t="inlineStr">
         <is>
@@ -4017,7 +4017,7 @@
       </c>
       <c r="B9" s="33">
         <f>-Datos!$B$53</f>
-        <v/>
+        <v>-48000.0</v>
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
@@ -4033,7 +4033,7 @@
       </c>
       <c r="B10" s="27">
         <f>B7+B8+B9</f>
-        <v/>
+        <v>-154800.0</v>
       </c>
       <c r="C10" s="29" t="n"/>
       <c r="D10" s="29" t="n"/>
@@ -4060,7 +4060,7 @@
       </c>
       <c r="B13" s="18">
         <f>Datos!$B$14*Datos!$B$15*Datos!$B$17/365</f>
-        <v/>
+        <v>443835.61643835617</v>
       </c>
       <c r="F13" s="9" t="inlineStr">
         <is>
@@ -4076,7 +4076,7 @@
       </c>
       <c r="B14" s="18">
         <f>Datos!$B$18*Escandallo!$D$10</f>
-        <v/>
+        <v>10520.0</v>
       </c>
       <c r="F14" s="9" t="inlineStr">
         <is>
@@ -4092,7 +4092,7 @@
       </c>
       <c r="B15" s="38">
         <f>B13+B14</f>
-        <v/>
+        <v>454355.61643835617</v>
       </c>
     </row>
     <row r="16">
@@ -4103,7 +4103,7 @@
       </c>
       <c r="B16" s="38">
         <f>-B15*Datos!$B$11</f>
-        <v/>
+        <v>-34076.67123287671</v>
       </c>
       <c r="F16" s="9" t="inlineStr">
         <is>
@@ -4131,7 +4131,7 @@
       </c>
       <c r="B19" s="52">
         <f>Persan!$B$10+Persan!$B$16</f>
-        <v/>
+        <v>-188876.67123287672</v>
       </c>
       <c r="C19" s="36" t="n"/>
       <c r="D19" s="36" t="n"/>
@@ -4150,7 +4150,7 @@
       </c>
       <c r="B20" s="47">
         <f>Persan!$B$19/PyG2025!$B$19</f>
-        <v/>
+        <v>-0.676095242167483</v>
       </c>
       <c r="F20" s="9" t="inlineStr">
         <is>
@@ -4166,7 +4166,7 @@
       </c>
       <c r="B21" s="38">
         <f>Persan!$B$19*Datos!$B$16</f>
-        <v/>
+        <v>-944383.3561643836</v>
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
@@ -4182,7 +4182,7 @@
       </c>
       <c r="B22" s="38">
         <f>PyG2025!$B$19+Persan!$B$19</f>
-        <v/>
+        <v>90487.32876712328</v>
       </c>
       <c r="F22" s="9" t="inlineStr">
         <is>
@@ -4238,15 +4238,15 @@
       </c>
       <c r="B26" s="53">
         <f>Escandallo!$D$10</f>
-        <v/>
+        <v>10.52</v>
       </c>
       <c r="C26" s="40">
         <f>B26-Datos!$B$15</f>
-        <v/>
+        <v>0.5199999999999996</v>
       </c>
       <c r="D26" s="30">
         <f>B26/Datos!$B$15-1</f>
-        <v/>
+        <v>0.052000000000000046</v>
       </c>
       <c r="F26" s="9" t="inlineStr">
         <is>
@@ -4262,15 +4262,15 @@
       </c>
       <c r="B27" s="53">
         <f>Escandallo!$D$10+(Datos!$B$50+Datos!$B$53)/Datos!$B$14</f>
-        <v/>
+        <v>11.719999999999999</v>
       </c>
       <c r="C27" s="40">
         <f>B27-Datos!$B$15</f>
-        <v/>
+        <v>1.7199999999999989</v>
       </c>
       <c r="D27" s="30">
         <f>B27/Datos!$B$15-1</f>
-        <v/>
+        <v>0.17199999999999993</v>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
@@ -4286,15 +4286,15 @@
       </c>
       <c r="B28" s="55">
         <f>(Datos!$B$14*Escandallo!$D$10+Datos!$B$50+Datos!$B$53)/(Datos!$B$14*(1-Datos!$B$17/365*Datos!$B$11))</f>
-        <v/>
+        <v>12.170128022759602</v>
       </c>
       <c r="C28" s="40">
         <f>B28-Datos!$B$15</f>
-        <v/>
+        <v>2.1701280227596023</v>
       </c>
       <c r="D28" s="30">
         <f>B28/Datos!$B$15-1</f>
-        <v/>
+        <v>0.21701280227596031</v>
       </c>
       <c r="F28" s="9" t="inlineStr">
         <is>
@@ -4310,15 +4310,15 @@
       </c>
       <c r="B29" s="53">
         <f>B27+Escandallo!$B$11</f>
-        <v/>
+        <v>14.51</v>
       </c>
       <c r="C29" s="40">
         <f>B29-Datos!$B$15</f>
-        <v/>
+        <v>4.51</v>
       </c>
       <c r="D29" s="30">
         <f>B29/Datos!$B$15-1</f>
-        <v/>
+        <v>0.45100000000000007</v>
       </c>
       <c r="F29" s="9" t="inlineStr">
         <is>
@@ -4372,15 +4372,15 @@
       </c>
       <c r="B33" s="40">
         <f>Escandallo!$D$6*(1+A33)+Escandallo!$D$7+Escandallo!$D$8+Escandallo!$D$9</f>
-        <v/>
+        <v>10.52</v>
       </c>
       <c r="C33" s="40">
         <f>Datos!$B$15-B33</f>
-        <v/>
+        <v>-0.5199999999999996</v>
       </c>
       <c r="D33" s="38">
         <f>C33*Datos!$B$14-Datos!$B$50-Datos!$B$53+Persan!$B$16</f>
-        <v/>
+        <v>-188876.6712328767</v>
       </c>
     </row>
     <row r="34">
@@ -4389,15 +4389,15 @@
       </c>
       <c r="B34" s="40">
         <f>Escandallo!$D$6*(1+A34)+Escandallo!$D$7+Escandallo!$D$8+Escandallo!$D$9</f>
-        <v/>
+        <v>10.9335</v>
       </c>
       <c r="C34" s="40">
         <f>Datos!$B$15-B34</f>
-        <v/>
+        <v>-0.9335000000000004</v>
       </c>
       <c r="D34" s="38">
         <f>C34*Datos!$B$14-Datos!$B$50-Datos!$B$53+Persan!$B$16</f>
-        <v/>
+        <v>-226091.67123287678</v>
       </c>
     </row>
     <row r="35">
@@ -4406,15 +4406,15 @@
       </c>
       <c r="B35" s="40">
         <f>Escandallo!$D$6*(1+A35)+Escandallo!$D$7+Escandallo!$D$8+Escandallo!$D$9</f>
-        <v/>
+        <v>11.347</v>
       </c>
       <c r="C35" s="40">
         <f>Datos!$B$15-B35</f>
-        <v/>
+        <v>-1.3469999999999995</v>
       </c>
       <c r="D35" s="38">
         <f>C35*Datos!$B$14-Datos!$B$50-Datos!$B$53+Persan!$B$16</f>
-        <v/>
+        <v>-263306.67123287666</v>
       </c>
     </row>
     <row r="36">
@@ -4423,15 +4423,15 @@
       </c>
       <c r="B36" s="40">
         <f>Escandallo!$D$6*(1+A36)+Escandallo!$D$7+Escandallo!$D$8+Escandallo!$D$9</f>
-        <v/>
+        <v>11.760499999999999</v>
       </c>
       <c r="C36" s="40">
         <f>Datos!$B$15-B36</f>
-        <v/>
+        <v>-1.7604999999999986</v>
       </c>
       <c r="D36" s="38">
         <f>C36*Datos!$B$14-Datos!$B$50-Datos!$B$53+Persan!$B$16</f>
-        <v/>
+        <v>-300521.6712328766</v>
       </c>
     </row>
     <row r="37">
@@ -4440,15 +4440,15 @@
       </c>
       <c r="B37" s="40">
         <f>Escandallo!$D$6*(1+A37)+Escandallo!$D$7+Escandallo!$D$8+Escandallo!$D$9</f>
-        <v/>
+        <v>12.174</v>
       </c>
       <c r="C37" s="40">
         <f>Datos!$B$15-B37</f>
-        <v/>
+        <v>-2.1739999999999995</v>
       </c>
       <c r="D37" s="38">
         <f>C37*Datos!$B$14-Datos!$B$50-Datos!$B$53+Persan!$B$16</f>
-        <v/>
+        <v>-337736.67123287666</v>
       </c>
     </row>
     <row r="38">
@@ -4478,7 +4478,7 @@
       </c>
       <c r="B41" s="56">
         <f>Datos!$B$60</f>
-        <v/>
+        <v>12.5</v>
       </c>
       <c r="F41" s="9" t="inlineStr">
         <is>
@@ -4494,7 +4494,7 @@
       </c>
       <c r="B42" s="45">
         <f>Datos!$B$61</f>
-        <v/>
+        <v>90.0</v>
       </c>
     </row>
     <row r="43">
@@ -4505,7 +4505,7 @@
       </c>
       <c r="B43" s="53">
         <f>B41-Escandallo!$D$10</f>
-        <v/>
+        <v>1.9800000000000004</v>
       </c>
     </row>
     <row r="44">
@@ -4516,7 +4516,7 @@
       </c>
       <c r="B44" s="18">
         <f>B43*Datos!$B$14</f>
-        <v/>
+        <v>178200.00000000003</v>
       </c>
     </row>
     <row r="45">
@@ -4527,7 +4527,7 @@
       </c>
       <c r="B45" s="18">
         <f>-Datos!$B$50-Datos!$B$53</f>
-        <v/>
+        <v>-108000.0</v>
       </c>
     </row>
     <row r="46">
@@ -4538,7 +4538,7 @@
       </c>
       <c r="B46" s="18">
         <f>-(B41*Datos!$B$14*B42/365+Datos!$B$18*Escandallo!$D$10)*Datos!$B$11</f>
-        <v/>
+        <v>-21593.794520547945</v>
       </c>
     </row>
     <row r="47">
@@ -4549,7 +4549,7 @@
       </c>
       <c r="B47" s="58">
         <f>B44+B45+B46</f>
-        <v/>
+        <v>48606.20547945208</v>
       </c>
       <c r="C47" s="59" t="n"/>
       <c r="D47" s="59" t="n"/>
@@ -4568,7 +4568,7 @@
       </c>
       <c r="B48" s="38">
         <f>B47-Persan!$B$19</f>
-        <v/>
+        <v>237482.8767123288</v>
       </c>
     </row>
   </sheetData>
@@ -4655,15 +4655,15 @@
       </c>
       <c r="B6" s="14">
         <f>Datos!$B$32</f>
-        <v/>
+        <v>500.0</v>
       </c>
       <c r="C6" s="14">
         <f>Datos!$B$21*Datos!$B$22*Datos!$B$8</f>
-        <v/>
+        <v>390.0</v>
       </c>
       <c r="D6" s="14">
         <f>Datos!$B$43*Datos!$B$44</f>
-        <v/>
+        <v>360.0</v>
       </c>
     </row>
     <row r="7">
@@ -4674,15 +4674,15 @@
       </c>
       <c r="B7" s="14">
         <f>Datos!$B$31</f>
-        <v/>
+        <v>8.0</v>
       </c>
       <c r="C7" s="14">
         <f>Datos!$B$23</f>
-        <v/>
+        <v>2.0</v>
       </c>
       <c r="D7" s="14">
         <f>Datos!$B$45</f>
-        <v/>
+        <v>1.0</v>
       </c>
     </row>
     <row r="8">
@@ -4693,15 +4693,15 @@
       </c>
       <c r="B8" s="20">
         <f>B6/B7</f>
-        <v/>
+        <v>62.5</v>
       </c>
       <c r="C8" s="20">
         <f>C6/C7</f>
-        <v/>
+        <v>195.0</v>
       </c>
       <c r="D8" s="20">
         <f>D6/D7</f>
-        <v/>
+        <v>360.0</v>
       </c>
       <c r="F8" s="9" t="inlineStr">
         <is>
@@ -4717,11 +4717,11 @@
       </c>
       <c r="C9" s="20">
         <f>Datos!$B$28</f>
-        <v/>
+        <v>6.0</v>
       </c>
       <c r="D9" s="20">
         <f>Datos!$B$46/60</f>
-        <v/>
+        <v>0.4166666666666667</v>
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
@@ -4737,15 +4737,15 @@
       </c>
       <c r="B10" s="40">
         <f>Datos!$B$9*B7/(B6*Datos!$B$7)</f>
-        <v/>
+        <v>2.512396694214876</v>
       </c>
       <c r="C10" s="40">
         <f>Datos!$B$9*C7/(C6*Datos!$B$7)</f>
-        <v/>
+        <v>0.8052553507098962</v>
       </c>
       <c r="D10" s="40">
         <f>Datos!$B$9*D7/(D6*Datos!$B$7)</f>
-        <v/>
+        <v>0.4361799816345271</v>
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
@@ -4773,7 +4773,7 @@
       </c>
       <c r="B13" s="45">
         <f>Capacidad!$B$18</f>
-        <v/>
+        <v>87120.0</v>
       </c>
     </row>
     <row r="14">
@@ -4784,7 +4784,7 @@
       </c>
       <c r="B14" s="20">
         <f>B13/(Datos!$B$33*Datos!$B$7)</f>
-        <v/>
+        <v>5.76</v>
       </c>
       <c r="F14" s="9" t="inlineStr">
         <is>
@@ -4800,7 +4800,7 @@
       </c>
       <c r="B15" s="45">
         <f>Datos!$B$45</f>
-        <v/>
+        <v>1.0</v>
       </c>
     </row>
     <row r="16">
@@ -4811,7 +4811,7 @@
       </c>
       <c r="B16" s="50">
         <f>B14-B15</f>
-        <v/>
+        <v>4.76</v>
       </c>
     </row>
     <row r="17">
@@ -4822,7 +4822,7 @@
       </c>
       <c r="B17" s="38">
         <f>B16*Datos!$B$9</f>
-        <v/>
+        <v>180880.0</v>
       </c>
       <c r="F17" s="9" t="inlineStr">
         <is>
@@ -4838,7 +4838,7 @@
       </c>
       <c r="B18" s="18">
         <f>-Datos!$B$42*(Datos!$B$11/12)/(1-(1+Datos!$B$11/12)^(-Datos!$B$54*12))*12</f>
-        <v/>
+        <v>-9618.215325899295</v>
       </c>
       <c r="F18" s="9" t="inlineStr">
         <is>
@@ -4854,7 +4854,7 @@
       </c>
       <c r="B19" s="38">
         <f>B17+B18</f>
-        <v/>
+        <v>171261.7846741007</v>
       </c>
     </row>
     <row r="20">
@@ -4865,7 +4865,7 @@
       </c>
       <c r="B20" s="50">
         <f>Datos!$B$42/B17*12</f>
-        <v/>
+        <v>2.6536930561698364</v>
       </c>
       <c r="F20" s="9" t="inlineStr">
         <is>
@@ -4900,7 +4900,7 @@
       </c>
       <c r="B25" s="61">
         <f>Datos!$B$59</f>
-        <v/>
+        <v>0.0</v>
       </c>
       <c r="F25" s="9" t="inlineStr">
         <is>
@@ -4916,7 +4916,7 @@
       </c>
       <c r="B26" s="38">
         <f>Robot!$B$17*Datos!$B$59</f>
-        <v/>
+        <v>0.0</v>
       </c>
     </row>
     <row r="27">
@@ -4927,7 +4927,7 @@
       </c>
       <c r="B27" s="33">
         <f>B18</f>
-        <v/>
+        <v>-9618.215325899295</v>
       </c>
     </row>
     <row r="28">
@@ -4938,7 +4938,7 @@
       </c>
       <c r="B28" s="38">
         <f>B26+B27</f>
-        <v/>
+        <v>-9618.215325899295</v>
       </c>
       <c r="F28" s="9" t="inlineStr">
         <is>
@@ -5010,19 +5010,19 @@
       </c>
       <c r="B33" s="56">
         <f>Datos!$B$15</f>
-        <v/>
+        <v>10.0</v>
       </c>
       <c r="C33" s="40">
         <f>Escandallo!$D$6+Escandallo!$D$7+Escandallo!$D$8+Escandallo!$D$9</f>
-        <v/>
+        <v>10.52</v>
       </c>
       <c r="D33" s="53">
         <f>B33-C33</f>
-        <v/>
+        <v>-0.5199999999999996</v>
       </c>
       <c r="E33" s="38">
         <f>D33*Capacidad!$B$18</f>
-        <v/>
+        <v>-45302.399999999965</v>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
@@ -5038,19 +5038,19 @@
       </c>
       <c r="B34" s="56">
         <f>Escandallo!$B$5</f>
-        <v/>
+        <v>15.16</v>
       </c>
       <c r="C34" s="40">
         <f>Escandallo!$D$6+Escandallo!$D$7+Escandallo!$D$8+Escandallo!$D$9</f>
-        <v/>
+        <v>10.52</v>
       </c>
       <c r="D34" s="53">
         <f>B34-C34</f>
-        <v/>
+        <v>4.640000000000001</v>
       </c>
       <c r="E34" s="38">
         <f>D34*Capacidad!$B$18</f>
-        <v/>
+        <v>404236.80000000005</v>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
@@ -5066,19 +5066,19 @@
       </c>
       <c r="B35" s="56">
         <f>Datos!$B$60</f>
-        <v/>
+        <v>12.5</v>
       </c>
       <c r="C35" s="40">
         <f>Escandallo!$D$6+Escandallo!$D$7+Escandallo!$D$8+Escandallo!$D$9</f>
-        <v/>
+        <v>10.52</v>
       </c>
       <c r="D35" s="53">
         <f>B35-C35</f>
-        <v/>
+        <v>1.9800000000000004</v>
       </c>
       <c r="E35" s="38">
         <f>D35*Capacidad!$B$18</f>
-        <v/>
+        <v>172497.60000000003</v>
       </c>
       <c r="F35" s="9" t="inlineStr">
         <is>
@@ -5094,7 +5094,7 @@
       </c>
       <c r="B36" s="52">
         <f>E34-E33</f>
-        <v/>
+        <v>449539.2</v>
       </c>
       <c r="C36" s="36" t="n"/>
       <c r="D36" s="36" t="n"/>
@@ -5192,7 +5192,7 @@
       </c>
       <c r="C5" s="18">
         <f>Datos!$B$55</f>
-        <v/>
+        <v>190000.0</v>
       </c>
       <c r="D5" s="18" t="inlineStr">
         <is>
@@ -5201,11 +5201,11 @@
       </c>
       <c r="E5" s="18">
         <f>Datos!$B$42</f>
-        <v/>
+        <v>40000.0</v>
       </c>
       <c r="F5" s="18">
         <f>Datos!$B$55</f>
-        <v/>
+        <v>190000.0</v>
       </c>
       <c r="G5" s="9" t="inlineStr">
         <is>
@@ -5226,7 +5226,7 @@
       </c>
       <c r="C6" s="14">
         <f>Datos!$B$14</f>
-        <v/>
+        <v>90000.0</v>
       </c>
       <c r="D6" s="14" t="inlineStr">
         <is>
@@ -5240,7 +5240,7 @@
       </c>
       <c r="F6" s="14">
         <f>Datos!$B$14</f>
-        <v/>
+        <v>90000.0</v>
       </c>
       <c r="G6" s="9" t="inlineStr">
         <is>
@@ -5261,7 +5261,7 @@
       </c>
       <c r="C7" s="18">
         <f>Persan!$B$7</f>
-        <v/>
+        <v>-46800.0</v>
       </c>
       <c r="D7" s="18" t="inlineStr">
         <is>
@@ -5275,7 +5275,7 @@
       </c>
       <c r="F7" s="18">
         <f>(Datos!$B$60-Escandallo!$D$10)*Datos!$B$14</f>
-        <v/>
+        <v>178200.00000000003</v>
       </c>
     </row>
     <row r="8">
@@ -5301,7 +5301,7 @@
       </c>
       <c r="E8" s="18">
         <f>Robot!$B$17*Datos!$B$59</f>
-        <v/>
+        <v>0.0</v>
       </c>
       <c r="F8" s="18" t="inlineStr">
         <is>
@@ -5327,7 +5327,7 @@
       </c>
       <c r="C9" s="18">
         <f>-Datos!$B$50</f>
-        <v/>
+        <v>-60000.0</v>
       </c>
       <c r="D9" s="18" t="inlineStr">
         <is>
@@ -5341,7 +5341,7 @@
       </c>
       <c r="F9" s="18">
         <f>-Datos!$B$50</f>
-        <v/>
+        <v>-60000.0</v>
       </c>
     </row>
     <row r="10">
@@ -5357,7 +5357,7 @@
       </c>
       <c r="C10" s="18">
         <f>-Datos!$B$53</f>
-        <v/>
+        <v>-48000.0</v>
       </c>
       <c r="D10" s="18" t="inlineStr">
         <is>
@@ -5366,11 +5366,11 @@
       </c>
       <c r="E10" s="18">
         <f>-Datos!$B$42*(Datos!$B$11/12)/(1-(1+Datos!$B$11/12)^(-Datos!$B$54*12))*12</f>
-        <v/>
+        <v>-9618.215325899295</v>
       </c>
       <c r="F10" s="18">
         <f>-Datos!$B$53</f>
-        <v/>
+        <v>-48000.0</v>
       </c>
       <c r="G10" s="9" t="inlineStr">
         <is>
@@ -5391,7 +5391,7 @@
       </c>
       <c r="C11" s="18">
         <f>Persan!$B$16</f>
-        <v/>
+        <v>-34076.67123287671</v>
       </c>
       <c r="D11" s="18" t="inlineStr">
         <is>
@@ -5405,7 +5405,7 @@
       </c>
       <c r="F11" s="18">
         <f>-(Datos!$B$60*Datos!$B$14*Datos!$B$61/365+Datos!$B$18*Escandallo!$D$10)*Datos!$B$11</f>
-        <v/>
+        <v>-21593.794520547945</v>
       </c>
       <c r="G11" s="9" t="inlineStr">
         <is>
@@ -5421,23 +5421,23 @@
       </c>
       <c r="B12" s="27">
         <f>SUM(B7:B11)</f>
-        <v/>
+        <v>0.0</v>
       </c>
       <c r="C12" s="27">
         <f>SUM(C7:C11)</f>
-        <v/>
+        <v>-188876.67123287672</v>
       </c>
       <c r="D12" s="27">
         <f>SUM(D7:D11)</f>
-        <v/>
+        <v>0.0</v>
       </c>
       <c r="E12" s="27">
         <f>SUM(E7:E11)</f>
-        <v/>
+        <v>-9618.215325899295</v>
       </c>
       <c r="F12" s="27">
         <f>SUM(F7:F11)</f>
-        <v/>
+        <v>48606.20547945208</v>
       </c>
       <c r="G12" s="29" t="n"/>
     </row>
@@ -5449,23 +5449,23 @@
       </c>
       <c r="B13" s="27">
         <f>PyG2025!$B$19+B12</f>
-        <v/>
+        <v>279364.0</v>
       </c>
       <c r="C13" s="27">
         <f>PyG2025!$B$19+C12</f>
-        <v/>
+        <v>90487.32876712328</v>
       </c>
       <c r="D13" s="27">
         <f>PyG2025!$B$19+D12</f>
-        <v/>
+        <v>279364.0</v>
       </c>
       <c r="E13" s="27">
         <f>PyG2025!$B$19+E12</f>
-        <v/>
+        <v>269745.7846741007</v>
       </c>
       <c r="F13" s="27">
         <f>PyG2025!$B$19+F12</f>
-        <v/>
+        <v>327970.2054794521</v>
       </c>
       <c r="G13" s="42" t="inlineStr">
         <is>
@@ -5481,23 +5481,23 @@
       </c>
       <c r="B14" s="30">
         <f>B12/PyG2025!$B$19</f>
-        <v/>
+        <v>0.0</v>
       </c>
       <c r="C14" s="30">
         <f>C12/PyG2025!$B$19</f>
-        <v/>
+        <v>-0.676095242167483</v>
       </c>
       <c r="D14" s="30">
         <f>D12/PyG2025!$B$19</f>
-        <v/>
+        <v>0.0</v>
       </c>
       <c r="E14" s="30">
         <f>E12/PyG2025!$B$19</f>
-        <v/>
+        <v>-0.03442897197169032</v>
       </c>
       <c r="F14" s="30">
         <f>F12/PyG2025!$B$19</f>
-        <v/>
+        <v>0.17398879411610688</v>
       </c>
     </row>
     <row r="16">
@@ -5521,23 +5521,23 @@
       </c>
       <c r="B17" s="18">
         <f>B12</f>
-        <v/>
+        <v>0.0</v>
       </c>
       <c r="C17" s="18">
         <f>C12</f>
-        <v/>
+        <v>-188876.67123287672</v>
       </c>
       <c r="D17" s="18">
         <f>D12</f>
-        <v/>
+        <v>0.0</v>
       </c>
       <c r="E17" s="18">
         <f>E12</f>
-        <v/>
+        <v>-9618.215325899295</v>
       </c>
       <c r="F17" s="18">
         <f>F12</f>
-        <v/>
+        <v>48606.20547945208</v>
       </c>
     </row>
     <row r="18">
@@ -5553,7 +5553,7 @@
       </c>
       <c r="C18" s="18">
         <f>-(Datos!$B$14*Datos!$B$15*Datos!$B$17/365+Datos!$B$18*Escandallo!$D$10)</f>
-        <v/>
+        <v>-454355.61643835617</v>
       </c>
       <c r="D18" s="18" t="inlineStr">
         <is>
@@ -5567,7 +5567,7 @@
       </c>
       <c r="F18" s="18">
         <f>-(Datos!$B$60*Datos!$B$14*Datos!$B$61/365+Datos!$B$18*Escandallo!$D$10)</f>
-        <v/>
+        <v>-287917.2602739726</v>
       </c>
       <c r="G18" s="9" t="inlineStr">
         <is>
@@ -5593,7 +5593,7 @@
       </c>
       <c r="D19" s="18">
         <f>-Datos!$B$63</f>
-        <v/>
+        <v>-200000.0</v>
       </c>
       <c r="E19" s="18" t="inlineStr">
         <is>
@@ -5619,23 +5619,23 @@
       </c>
       <c r="B20" s="35">
         <f>SUM(B17:B19)</f>
-        <v/>
+        <v>0.0</v>
       </c>
       <c r="C20" s="35">
         <f>SUM(C17:C19)</f>
-        <v/>
+        <v>-643232.2876712328</v>
       </c>
       <c r="D20" s="35">
         <f>SUM(D17:D19)</f>
-        <v/>
+        <v>-200000.0</v>
       </c>
       <c r="E20" s="35">
         <f>SUM(E17:E19)</f>
-        <v/>
+        <v>-9618.215325899295</v>
       </c>
       <c r="F20" s="35">
         <f>SUM(F17:F19)</f>
-        <v/>
+        <v>-239311.0547945205</v>
       </c>
       <c r="G20" s="37" t="inlineStr">
         <is>
@@ -5651,7 +5651,7 @@
       </c>
       <c r="B21" s="33">
         <f>PyG2025!$B$31</f>
-        <v/>
+        <v>-60555.0</v>
       </c>
     </row>
     <row r="23">

</xml_diff>